<commit_message>
Adição de restaurante na base
</commit_message>
<xml_diff>
--- a/dados/base_cnpjs.xlsx
+++ b/dados/base_cnpjs.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2337" uniqueCount="2281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="2284">
   <si>
     <t xml:space="preserve">SIGLA</t>
   </si>
@@ -6863,6 +6863,15 @@
   </si>
   <si>
     <t xml:space="preserve">ZZZ - MCDONALDS - CASCAVEL DRIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DBV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42591651264124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DBV MCDONALDS CULTURA</t>
   </si>
 </sst>
 </file>
@@ -6983,8 +6992,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C779"/>
+  <dimension ref="A1:C780"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="59.35"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -15553,6 +15566,17 @@
       </c>
       <c r="C779" s="2" t="s">
         <v>2280</v>
+      </c>
+    </row>
+    <row r="780" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A780" s="0" t="s">
+        <v>2281</v>
+      </c>
+      <c r="B780" s="2" t="s">
+        <v>2282</v>
+      </c>
+      <c r="C780" s="0" t="s">
+        <v>2283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>